<commit_message>
feat: complete multi-agent hierarchy, entity system, durable harness & concurrency safe I/O
</commit_message>
<xml_diff>
--- a/users/input/AnPT/entities-FPA-AnPT.xlsx
+++ b/users/input/AnPT/entities-FPA-AnPT.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
   <si>
     <t>tickers</t>
   </si>
@@ -29,6 +29,21 @@
     <t>industries</t>
   </si>
   <si>
+    <t>nations</t>
+  </si>
+  <si>
+    <t>themes</t>
+  </si>
+  <si>
+    <t>macro</t>
+  </si>
+  <si>
+    <t>assets</t>
+  </si>
+  <si>
+    <t>institutions</t>
+  </si>
+  <si>
     <t>entities</t>
   </si>
   <si>
@@ -47,6 +62,18 @@
     <t>THEP</t>
   </si>
   <si>
+    <t>MY</t>
+  </si>
+  <si>
+    <t>LAM_PHAT</t>
+  </si>
+  <si>
+    <t>CO_PHIEU</t>
+  </si>
+  <si>
+    <t>FED</t>
+  </si>
+  <si>
     <t>FPT</t>
   </si>
   <si>
@@ -59,6 +86,18 @@
     <t>NGAN_HANG</t>
   </si>
   <si>
+    <t>TRUNG_QUOC</t>
+  </si>
+  <si>
+    <t>DAU_TU_CONG</t>
+  </si>
+  <si>
+    <t>VANG</t>
+  </si>
+  <si>
+    <t>NHNN</t>
+  </si>
+  <si>
     <t>VCB</t>
   </si>
   <si>
@@ -71,6 +110,15 @@
     <t>DAU_KHI</t>
   </si>
   <si>
+    <t>NANG_HANG_TTCK</t>
+  </si>
+  <si>
+    <t>TIEN_MA_HOA</t>
+  </si>
+  <si>
+    <t>UBCKNN</t>
+  </si>
+  <si>
     <t>VNM</t>
   </si>
   <si>
@@ -78,6 +126,9 @@
   </si>
   <si>
     <t>QUY</t>
+  </si>
+  <si>
+    <t>HANG_HOA_NONG_SAN</t>
   </si>
   <si>
     <t>MWG</t>
@@ -517,13 +568,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -542,134 +593,185 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="F2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+      <c r="G4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I4" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="C5" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>37</v>
+      </c>
+      <c r="I5" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>33</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>35</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -688,26 +790,26 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="B1" t="s">
-        <v>38</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>58</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -918,13 +1020,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08ADE00B-913D-4D1D-8C04-872D1EB82DE6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32D48E68-9DA9-4A20-B99C-B51C472B4027}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2741A813-26D2-4B37-9D21-A97CD23D2B11}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BE62501F-7EBC-4A13-8BC4-0C571F066CA2}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B003704D-2E7E-40EC-A8DA-4914BA2ABCF3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28044DF9-6F04-4C80-8C0F-256675B61965}"/>
 </file>
</xml_diff>